<commit_message>
Add Bermudan swaption example
</commit_message>
<xml_diff>
--- a/tests/workbooks/test_gaussian1dmodel.xlsx
+++ b/tests/workbooks/test_gaussian1dmodel.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BEE558A-B37D-4A08-A81C-F0469726BDD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2FC726-D8B8-4AD7-8809-B6520A5E18F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3570" yWindow="-19950" windowWidth="33045" windowHeight="18270" xr2:uid="{096EF196-26B4-4940-94D5-2518E57D2FCB}"/>
+    <workbookView xWindow="-120" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{096EF196-26B4-4940-94D5-2518E57D2FCB}"/>
   </bookViews>
   <sheets>
     <sheet name="GSR Model and Engine" sheetId="1" r:id="rId1"/>
+    <sheet name="Bermudan Swaption" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -61,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="109">
   <si>
     <t>Evaluation date</t>
   </si>
@@ -256,12 +257,147 @@
   </si>
   <si>
     <t>qlGsrReversion</t>
+  </si>
+  <si>
+    <t>Projection curve</t>
+  </si>
+  <si>
+    <t>Discount curve</t>
+  </si>
+  <si>
+    <t>Expiry | Swap term</t>
+  </si>
+  <si>
+    <t>3y</t>
+  </si>
+  <si>
+    <t>4y</t>
+  </si>
+  <si>
+    <t>6y</t>
+  </si>
+  <si>
+    <t>7y</t>
+  </si>
+  <si>
+    <t>8y</t>
+  </si>
+  <si>
+    <t>9y</t>
+  </si>
+  <si>
+    <t>10y</t>
+  </si>
+  <si>
+    <t>Expiry dates</t>
+  </si>
+  <si>
+    <t>(Normal) VolTS</t>
+  </si>
+  <si>
+    <t>Swap start</t>
+  </si>
+  <si>
+    <t>Swap length</t>
+  </si>
+  <si>
+    <t>Effective date</t>
+  </si>
+  <si>
+    <t>Spot lag</t>
+  </si>
+  <si>
+    <t>2d</t>
+  </si>
+  <si>
+    <t>Calendar</t>
+  </si>
+  <si>
+    <t>TARGET</t>
+  </si>
+  <si>
+    <t>Maturity date</t>
+  </si>
+  <si>
+    <t>Day count</t>
+  </si>
+  <si>
+    <t>Exercise</t>
+  </si>
+  <si>
+    <t>Fixed leg idx</t>
+  </si>
+  <si>
+    <t>Exercse date</t>
+  </si>
+  <si>
+    <t>Bermudan exercise</t>
+  </si>
+  <si>
+    <t>European swaption 1y</t>
+  </si>
+  <si>
+    <t>European swaption 3y</t>
+  </si>
+  <si>
+    <t>European swaption 5y</t>
+  </si>
+  <si>
+    <t>European swaption 7y</t>
+  </si>
+  <si>
+    <t>European swaption 9y</t>
+  </si>
+  <si>
+    <t>Calibration helper</t>
+  </si>
+  <si>
+    <t>GSR model</t>
+  </si>
+  <si>
+    <t>Engine</t>
+  </si>
+  <si>
+    <t>Set engine</t>
+  </si>
+  <si>
+    <t>Optimization method</t>
+  </si>
+  <si>
+    <t>End criteria</t>
+  </si>
+  <si>
+    <t>Implied volatility</t>
+  </si>
+  <si>
+    <t>Initial GSR vol</t>
+  </si>
+  <si>
+    <t>GSR mean rev.</t>
+  </si>
+  <si>
+    <t>GSR vol</t>
+  </si>
+  <si>
+    <t>Calibrate volatility</t>
+  </si>
+  <si>
+    <t>NPV</t>
+  </si>
+  <si>
+    <t>Switch value</t>
+  </si>
+  <si>
+    <t>GSR mean reversion</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000%"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -315,7 +451,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -342,6 +478,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -681,7 +827,8 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="35.33203125" customWidth="1"/>
+    <col min="3" max="5" width="24.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -707,7 +854,7 @@
       </c>
       <c r="B4" t="str" cm="1">
         <f t="array" ref="B4">_xll.qlFlatForward(B2,0.03,"Act/365")</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R4C2YieldTermStructureHandle,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R4C2YieldTermStructureHandle,A</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -776,7 +923,7 @@
       </c>
       <c r="B13" t="str" cm="1">
         <f t="array" ref="B13">_xll.qlGsr(B4,B8:D8,B9:E9,B10:E10,B11)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R13C2Gsr,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R13C2Gsr,A</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -785,7 +932,7 @@
       </c>
       <c r="B15" t="str" cm="1">
         <f t="array" ref="B15">_xll.qlGaussian1dSwaptionEngine(B13)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R15C2Gaussian1dSwaptionEngine,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R15C2Gaussian1dSwaptionEngine,A</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -794,7 +941,7 @@
       </c>
       <c r="B17" s="4" t="str" cm="1">
         <f t="array" ref="B17">_xll.qlFlatForward(B2,0.03)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R17C2YieldTermStructureHandle,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R17C2YieldTermStructureHandle,A</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -803,7 +950,7 @@
       </c>
       <c r="B18" s="4" t="str" cm="1">
         <f t="array" ref="B18">_xll.qlEuribor("6M",B17)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R18C2Euribor,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R18C2Euribor,A</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -857,7 +1004,7 @@
       </c>
       <c r="B25" s="4" t="str" cm="1">
         <f t="array" ref="B25">_xll.qlMakeSchedule(B22,B23,"1y",,"Target","ModifiedFollowing",,"Backward")</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R25C2Schedule,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R25C2Schedule,A</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
@@ -866,7 +1013,7 @@
       </c>
       <c r="B26" s="4" t="str" cm="1">
         <f t="array" ref="B26">_xll.qlMakeSchedule(B22,B23,"6m",,"Target","ModifiedFollowing",,"Backward")</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R26C2Schedule,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R26C2Schedule,A</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
@@ -875,7 +1022,7 @@
       </c>
       <c r="B27" s="4" t="str" cm="1">
         <f t="array" ref="B27">_xll.qlVanillaSwap("Payer",10000,B25,B24,"30/360",B26,B18,0,"Act/360")</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R27C2VanillaSwap,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R27C2VanillaSwap,A</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
@@ -919,7 +1066,7 @@
       </c>
       <c r="B35" s="4" t="str" cm="1">
         <f t="array" ref="B35">_xll.qlEuropeanExercise(B29)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R35C2EuropeanExercise,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R35C2EuropeanExercise,A</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
@@ -928,7 +1075,7 @@
       </c>
       <c r="B36" s="4" t="str" cm="1">
         <f t="array" ref="B36">_xll.qlBermudanExercise(B29:B32)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R36C2BermudanExercise,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R36C2BermudanExercise,A</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
@@ -955,7 +1102,7 @@
       </c>
       <c r="B41" s="4" t="str" cm="1">
         <f t="array" ref="B41">_xll.qlSwaption(B27,B35)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R41C2Swaption,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R41C2Swaption,A</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
@@ -964,7 +1111,7 @@
       </c>
       <c r="B42" s="4" t="str" cm="1">
         <f t="array" ref="B42">_xll.qlSwaption(B27,B36)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R42C2Swaption,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R42C2Swaption,A</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
@@ -1056,19 +1203,19 @@
       </c>
       <c r="B52" s="4" t="str">
         <f>$B$18</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R18C2Euribor,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R18C2Euribor,A</v>
       </c>
       <c r="C52" s="4" t="str">
         <f>$B$18</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R18C2Euribor,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R18C2Euribor,A</v>
       </c>
       <c r="D52" s="4" t="str">
         <f>$B$18</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R18C2Euribor,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R18C2Euribor,A</v>
       </c>
       <c r="E52" s="4" t="str">
         <f>$B$18</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R18C2Euribor,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R18C2Euribor,A</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
@@ -1128,19 +1275,19 @@
       </c>
       <c r="B56" s="4" t="str">
         <f>$B$4</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R4C2YieldTermStructureHandle,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R4C2YieldTermStructureHandle,A</v>
       </c>
       <c r="C56" s="4" t="str">
         <f>$B$4</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R4C2YieldTermStructureHandle,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R4C2YieldTermStructureHandle,A</v>
       </c>
       <c r="D56" s="4" t="str">
         <f>$B$4</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R4C2YieldTermStructureHandle,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R4C2YieldTermStructureHandle,A</v>
       </c>
       <c r="E56" s="4" t="str">
         <f>$B$4</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R4C2YieldTermStructureHandle,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R4C2YieldTermStructureHandle,A</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
@@ -1268,19 +1415,19 @@
       </c>
       <c r="B65" s="4" t="str" cm="1">
         <f t="array" ref="B65">_xll.qlSwaptionHelper(B49,B50,B51,B52,B53,B54,B55,B56,B57,B58,B59,B60,B61,B62)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R65C2SwaptionHelper,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R65C2SwaptionHelper,A</v>
       </c>
       <c r="C65" s="4" t="str" cm="1">
         <f t="array" ref="C65">_xll.qlSwaptionHelper(C49,C50,C51,C52,C53,C54,C55,C56,C57,C58,C59,C60,C61,C62)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R65C3SwaptionHelper,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R65C3SwaptionHelper,A</v>
       </c>
       <c r="D65" s="4" t="str" cm="1">
         <f t="array" ref="D65">_xll.qlSwaptionHelper(D49,D50,D51,D52,D53,D54,D55,D56,D57,D58,D59,D60,D61,D62)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R65C4SwaptionHelper,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R65C4SwaptionHelper,A</v>
       </c>
       <c r="E65" s="4" t="str" cm="1">
         <f t="array" ref="E65">_xll.qlSwaptionHelper(E49,E50,E51,E52,E53,E54,E55,E56,E57,E58,E59,E60,E61,E62)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R65C5SwaptionHelper,A</v>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R65C5SwaptionHelper,A</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
@@ -1306,8 +1453,8 @@
         <v>55</v>
       </c>
       <c r="B68" t="str" cm="1">
-        <f t="array" ref="B68">_xll.qlLevenbergMarquardt()</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R68C2LevenbergMarquardt,A</v>
+        <f t="array" ref="B68">_xll.qlLevenbergMarquardt(,,,,B66:E66)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R68C2LevenbergMarquardt,A</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
@@ -1355,8 +1502,8 @@
         <v>61</v>
       </c>
       <c r="B75" t="str" cm="1">
-        <f t="array" ref="B75">_xll.qlEndCriteria(B70,B71,B72,B73,B74)</f>
-        <v>欣[test_gaussian1dmodel.xlsx]GSR Model and Engine!R75C2EndCriteria,A</v>
+        <f t="array" ref="B75">_xll.qlEndCriteria(B70,B71,B72,B73,B74,B66:E66)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]GSR Model and Engine!R75C2EndCriteria,A</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
@@ -1377,13 +1524,13 @@
         <v>6.9631874311834709E-3</v>
       </c>
       <c r="C79">
-        <v>6.9629046225871821E-3</v>
+        <v>6.9598377904623336E-3</v>
       </c>
       <c r="D79">
-        <v>6.9692329562232634E-3</v>
+        <v>6.9692472977811214E-3</v>
       </c>
       <c r="E79">
-        <v>6.9962829631992464E-3</v>
+        <v>6.9991762124002365E-3</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
@@ -1402,6 +1549,913 @@
       </c>
       <c r="E80">
         <v>0.01</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3DE146D-E077-4092-A23A-A651D070976A}">
+  <dimension ref="A1:X62"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.77734375" customWidth="1"/>
+    <col min="11" max="11" width="14.21875" customWidth="1"/>
+    <col min="15" max="15" width="14.77734375" customWidth="1"/>
+    <col min="16" max="16" width="12.109375" customWidth="1"/>
+    <col min="17" max="18" width="13.5546875" customWidth="1"/>
+    <col min="19" max="19" width="13.109375" customWidth="1"/>
+    <col min="20" max="20" width="18.5546875" customWidth="1"/>
+    <col min="21" max="21" width="15" customWidth="1"/>
+    <col min="22" max="22" width="13.21875" customWidth="1"/>
+    <col min="23" max="23" width="11.33203125" customWidth="1"/>
+    <col min="24" max="24" width="10.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" cm="1">
+        <f t="array" ref="B2">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="J4" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="N4" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="O4" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="P4" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q4" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="R4" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="S4" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="T4" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="U4" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="V4" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="W4" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="X4" s="12" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="D5" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="2">
+        <v>7.3156703444470991E-3</v>
+      </c>
+      <c r="F5" s="2">
+        <v>7.3545191823137079E-3</v>
+      </c>
+      <c r="G5" s="2">
+        <v>7.2034359041569691E-3</v>
+      </c>
+      <c r="H5" s="2">
+        <v>7.0085770171602179E-3</v>
+      </c>
+      <c r="I5" s="2">
+        <v>6.8685932674608981E-3</v>
+      </c>
+      <c r="J5" s="2">
+        <v>6.7945145206867591E-3</v>
+      </c>
+      <c r="K5" s="1" cm="1">
+        <f t="array" ref="K5">_xll.qlCalendarAdvance2($B$4,$B$2,D5)</f>
+        <v>46905</v>
+      </c>
+      <c r="L5" s="13"/>
+      <c r="O5" s="12">
+        <v>1</v>
+      </c>
+      <c r="P5" s="1" cm="1">
+        <f t="array" ref="P5">INDEX(_xll.qlScheduleDates($B$20),O5)</f>
+        <v>46541</v>
+      </c>
+      <c r="Q5" s="1" cm="1">
+        <f t="array" ref="Q5">_xll.qlCalendarAdvance2($B$4,P5,"-2d")</f>
+        <v>46539</v>
+      </c>
+      <c r="R5" s="14" t="str">
+        <f>(10-O5)&amp;"y"</f>
+        <v>9y</v>
+      </c>
+      <c r="S5" s="15" cm="1">
+        <f t="array" ref="S5">_xll.qlSwaptionVolatilityStructureVolatility($B$9,Q5,R5,$B$23)</f>
+        <v>6.8416161029777513E-3</v>
+      </c>
+      <c r="T5" s="4" t="str" cm="1">
+        <f t="array" ref="T5">_xll.qlSwaptionHelper(Q5,R5,S5,$B$11,"1y","30/360","act/360",$B$7,,$B$23,,"Normal",,2)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R5C20SwaptionHelper,A</v>
+      </c>
+      <c r="U5" s="13">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="V5" s="16">
+        <f>$B$39</f>
+        <v>0.03</v>
+      </c>
+      <c r="W5" t="b" cm="1">
+        <f t="array" ref="W5">_xll.qlBlackCalibrationHelperSetPricingEngine(T5,$B$41)</f>
+        <v>1</v>
+      </c>
+      <c r="X5" s="2" cm="1">
+        <f t="array" ref="X5:X10">_xll.qlGsrVolatility(B40,B52)</f>
+        <v>7.6211372531143793E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="4" t="str" cm="1">
+        <f t="array" ref="B6">_xll.qlFlatForward($B$2,0.03,"Act/365")</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R6C2YieldTermStructureHandle,A</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" s="2">
+        <v>7.3156703444470991E-3</v>
+      </c>
+      <c r="F6" s="2">
+        <v>7.3545191823137079E-3</v>
+      </c>
+      <c r="G6" s="2">
+        <v>7.2034359041569691E-3</v>
+      </c>
+      <c r="H6" s="2">
+        <v>7.0085770171602179E-3</v>
+      </c>
+      <c r="I6" s="2">
+        <v>6.8685932674608981E-3</v>
+      </c>
+      <c r="J6" s="2">
+        <v>6.7609933594352887E-3</v>
+      </c>
+      <c r="K6" s="1" cm="1">
+        <f t="array" ref="K6">_xll.qlCalendarAdvance2($B$4,$B$2,D6)</f>
+        <v>47270</v>
+      </c>
+      <c r="O6" s="12">
+        <v>3</v>
+      </c>
+      <c r="P6" s="1" cm="1">
+        <f t="array" ref="P6">INDEX(_xll.qlScheduleDates($B$20),O6)</f>
+        <v>47273</v>
+      </c>
+      <c r="Q6" s="1" cm="1">
+        <f t="array" ref="Q6">_xll.qlCalendarAdvance2($B$4,P6,"-2d")</f>
+        <v>47269</v>
+      </c>
+      <c r="R6" s="14" t="str">
+        <f t="shared" ref="R6:R9" si="0">(10-O6)&amp;"y"</f>
+        <v>7y</v>
+      </c>
+      <c r="S6" s="15" cm="1">
+        <f t="array" ref="S6">_xll.qlSwaptionVolatilityStructureVolatility($B$9,Q6,R6,$B$23)</f>
+        <v>6.8685932674608981E-3</v>
+      </c>
+      <c r="T6" s="4" t="str" cm="1">
+        <f t="array" ref="T6">_xll.qlSwaptionHelper(Q6,R6,S6,$B$11,"1y","30/360","act/360",$B$7,,$B$23,,"Normal",,2)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R6C20SwaptionHelper,A</v>
+      </c>
+      <c r="U6" s="13">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="V6" s="16">
+        <f t="shared" ref="V6:V10" si="1">$B$39</f>
+        <v>0.03</v>
+      </c>
+      <c r="W6" t="b" cm="1">
+        <f t="array" ref="W6">_xll.qlBlackCalibrationHelperSetPricingEngine(T6,$B$41)</f>
+        <v>1</v>
+      </c>
+      <c r="X6" s="2">
+        <v>7.7086247092700601E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="4" t="str" cm="1">
+        <f t="array" ref="B7">_xll.qlFlatForward($B$2,0.02,"Act/365")</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R7C2YieldTermStructureHandle,A</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="2">
+        <v>7.2817581863660278E-3</v>
+      </c>
+      <c r="F7" s="2">
+        <v>7.2696284121221786E-3</v>
+      </c>
+      <c r="G7" s="2">
+        <v>7.1304987601498587E-3</v>
+      </c>
+      <c r="H7" s="2">
+        <v>6.9283035181297286E-3</v>
+      </c>
+      <c r="I7" s="2">
+        <v>6.8008276595723591E-3</v>
+      </c>
+      <c r="J7" s="2">
+        <v>6.667429100858718E-3</v>
+      </c>
+      <c r="K7" s="1" cm="1">
+        <f t="array" ref="K7">_xll.qlCalendarAdvance2($B$4,$B$2,D7)</f>
+        <v>47637</v>
+      </c>
+      <c r="O7" s="12">
+        <v>5</v>
+      </c>
+      <c r="P7" s="1" cm="1">
+        <f t="array" ref="P7">INDEX(_xll.qlScheduleDates($B$20),O7)</f>
+        <v>48002</v>
+      </c>
+      <c r="Q7" s="1" cm="1">
+        <f t="array" ref="Q7">_xll.qlCalendarAdvance2($B$4,P7,"-2d")</f>
+        <v>47998</v>
+      </c>
+      <c r="R7" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>5y</v>
+      </c>
+      <c r="S7" s="15" cm="1">
+        <f t="array" ref="S7">_xll.qlSwaptionVolatilityStructureVolatility($B$9,Q7,R7,$B$23)</f>
+        <v>6.8308101938307384E-3</v>
+      </c>
+      <c r="T7" s="4" t="str" cm="1">
+        <f t="array" ref="T7">_xll.qlSwaptionHelper(Q7,R7,S7,$B$11,"1y","30/360","act/360",$B$7,,$B$23,,"Normal",,2)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R7C20SwaptionHelper,A</v>
+      </c>
+      <c r="U7" s="13">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="V7" s="16">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="W7" t="b" cm="1">
+        <f t="array" ref="W7">_xll.qlBlackCalibrationHelperSetPricingEngine(T7,$B$41)</f>
+        <v>1</v>
+      </c>
+      <c r="X7" s="2">
+        <v>7.5952162222992737E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="D8" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="2">
+        <v>7.2127847115574777E-3</v>
+      </c>
+      <c r="F8" s="2">
+        <v>7.2041310210440683E-3</v>
+      </c>
+      <c r="G8" s="2">
+        <v>7.0263612417479082E-3</v>
+      </c>
+      <c r="H8" s="2">
+        <v>6.8299999999999993E-3</v>
+      </c>
+      <c r="I8" s="2">
+        <v>6.7098768442212988E-3</v>
+      </c>
+      <c r="J8" s="2">
+        <v>6.5734245883187388E-3</v>
+      </c>
+      <c r="K8" s="1" cm="1">
+        <f t="array" ref="K8">_xll.qlCalendarAdvance2($B$4,$B$2,D8)</f>
+        <v>48001</v>
+      </c>
+      <c r="O8" s="12">
+        <v>7</v>
+      </c>
+      <c r="P8" s="1" cm="1">
+        <f t="array" ref="P8">INDEX(_xll.qlScheduleDates($B$20),O8)</f>
+        <v>48733</v>
+      </c>
+      <c r="Q8" s="1" cm="1">
+        <f t="array" ref="Q8">_xll.qlCalendarAdvance2($B$4,P8,"-2d")</f>
+        <v>48731</v>
+      </c>
+      <c r="R8" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>3y</v>
+      </c>
+      <c r="S8" s="15" cm="1">
+        <f t="array" ref="S8">_xll.qlSwaptionVolatilityStructureVolatility($B$9,Q8,R8,$B$23)</f>
+        <v>6.7802047066821882E-3</v>
+      </c>
+      <c r="T8" s="4" t="str" cm="1">
+        <f t="array" ref="T8">_xll.qlSwaptionHelper(Q8,R8,S8,$B$11,"1y","30/360","act/360",$B$7,,$B$23,,"Normal",,2)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R8C20SwaptionHelper,A</v>
+      </c>
+      <c r="U8" s="13">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="V8" s="16">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="W8" t="b" cm="1">
+        <f t="array" ref="W8">_xll.qlBlackCalibrationHelperSetPricingEngine(T8,$B$41)</f>
+        <v>1</v>
+      </c>
+      <c r="X8" s="2">
+        <v>7.4940275000552952E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="4" t="str" cm="1">
+        <f t="array" ref="B9">_xll.qlSwaptionVolatilityMatrix(B2,K5:K13,E4:J4,E5:J13,"act/365",,"Normal")</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R9C2SwaptionVolatilityStructureHandle,A</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" s="2">
+        <v>7.1067227208732493E-3</v>
+      </c>
+      <c r="F9" s="2">
+        <v>7.0954835416969491E-3</v>
+      </c>
+      <c r="G9" s="2">
+        <v>6.9032080676596688E-3</v>
+      </c>
+      <c r="H9" s="2">
+        <v>6.6952517114972181E-3</v>
+      </c>
+      <c r="I9" s="2">
+        <v>6.5607795355508477E-3</v>
+      </c>
+      <c r="J9" s="2">
+        <v>6.4205016338086587E-3</v>
+      </c>
+      <c r="K9" s="1" cm="1">
+        <f t="array" ref="K9">_xll.qlCalendarAdvance2($B$4,$B$2,D9)</f>
+        <v>48366</v>
+      </c>
+      <c r="O9" s="12">
+        <v>9</v>
+      </c>
+      <c r="P9" s="1" cm="1">
+        <f t="array" ref="P9">INDEX(_xll.qlScheduleDates($B$20),O9)</f>
+        <v>49464</v>
+      </c>
+      <c r="Q9" s="1" cm="1">
+        <f t="array" ref="Q9">_xll.qlCalendarAdvance2($B$4,P9,"-2d")</f>
+        <v>49460</v>
+      </c>
+      <c r="R9" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>1y</v>
+      </c>
+      <c r="S9" s="15" cm="1">
+        <f t="array" ref="S9">_xll.qlSwaptionVolatilityStructureVolatility($B$9,Q9,R9,$B$23)</f>
+        <v>6.7856340498962438E-3</v>
+      </c>
+      <c r="T9" s="4" t="str" cm="1">
+        <f t="array" ref="T9">_xll.qlSwaptionHelper(Q9,R9,S9,$B$11,"1y","30/360","act/360",$B$7,,$B$23,,"Normal",,2)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R9C20SwaptionHelper,A</v>
+      </c>
+      <c r="U9" s="13">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="V9" s="16">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="W9" t="b" cm="1">
+        <f t="array" ref="W9">_xll.qlBlackCalibrationHelperSetPricingEngine(T9,$B$41)</f>
+        <v>1</v>
+      </c>
+      <c r="X9" s="2">
+        <v>7.5255128544283187E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="D10" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" s="2">
+        <v>6.9935462562427386E-3</v>
+      </c>
+      <c r="F10" s="2">
+        <v>6.9834102491734378E-3</v>
+      </c>
+      <c r="G10" s="2">
+        <v>6.7802047066821882E-3</v>
+      </c>
+      <c r="H10" s="2">
+        <v>6.5598608899994481E-3</v>
+      </c>
+      <c r="I10" s="2">
+        <v>6.408766326632169E-3</v>
+      </c>
+      <c r="J10" s="2">
+        <v>6.2645776071992877E-3</v>
+      </c>
+      <c r="K10" s="1" cm="1">
+        <f t="array" ref="K10">_xll.qlCalendarAdvance2($B$4,$B$2,D10)</f>
+        <v>48731</v>
+      </c>
+      <c r="U10" s="13">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="V10" s="16">
+        <f t="shared" si="1"/>
+        <v>0.03</v>
+      </c>
+      <c r="X10" s="2">
+        <v>7.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="str" cm="1">
+        <f t="array" ref="B11">_xll.qlEuribor("6m",B6)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R11C2Euribor,A</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" s="2">
+        <v>6.8407381849624888E-3</v>
+      </c>
+      <c r="F11" s="2">
+        <v>6.8608351762795578E-3</v>
+      </c>
+      <c r="G11" s="2">
+        <v>6.6571986033943584E-3</v>
+      </c>
+      <c r="H11" s="2">
+        <v>6.4157223331967883E-3</v>
+      </c>
+      <c r="I11" s="2">
+        <v>6.2640620876668589E-3</v>
+      </c>
+      <c r="J11" s="2">
+        <v>6.0960353967729093E-3</v>
+      </c>
+      <c r="K11" s="1" cm="1">
+        <f t="array" ref="K11">_xll.qlCalendarAdvance2($B$4,$B$2,D11)</f>
+        <v>49096</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="D12" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="2">
+        <v>6.785482664909798E-3</v>
+      </c>
+      <c r="F12" s="2">
+        <v>6.7661093849715487E-3</v>
+      </c>
+      <c r="G12" s="2">
+        <v>6.554176344910399E-3</v>
+      </c>
+      <c r="H12" s="2">
+        <v>6.2951067334708986E-3</v>
+      </c>
+      <c r="I12" s="2">
+        <v>6.1192589232749693E-3</v>
+      </c>
+      <c r="J12" s="2">
+        <v>5.9343809605290482E-3</v>
+      </c>
+      <c r="K12" s="1" cm="1">
+        <f t="array" ref="K12">_xll.qlCalendarAdvance2($B$4,$B$2,D12)</f>
+        <v>49461</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E13" s="2">
+        <v>6.6471299594392692E-3</v>
+      </c>
+      <c r="F13" s="2">
+        <v>6.6550559406967393E-3</v>
+      </c>
+      <c r="G13" s="2">
+        <v>6.4498956923306483E-3</v>
+      </c>
+      <c r="H13" s="2">
+        <v>6.1746353255577487E-3</v>
+      </c>
+      <c r="I13" s="2">
+        <v>5.9884341705214589E-3</v>
+      </c>
+      <c r="J13" s="2">
+        <v>5.7827242854212382E-3</v>
+      </c>
+      <c r="K13" s="1" cm="1">
+        <f t="array" ref="K13">_xll.qlCalendarAdvance2($B$4,$B$2,D13)</f>
+        <v>49828</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="1" cm="1">
+        <f t="array" ref="B17">_xll.qlCalendarAdvance2($B$4,_xll.qlCalendarAdvance2($B$4,$B$2,$B$13),$B$15)</f>
+        <v>46541</v>
+      </c>
+      <c r="L17" s="1"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>84</v>
+      </c>
+      <c r="B18" s="1" cm="1">
+        <f t="array" ref="B18">_xll.qlCalendarAdvance2($B$4,$B$17,$B$14)</f>
+        <v>50194</v>
+      </c>
+      <c r="L18" s="1"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L19" s="1"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="4" t="str" cm="1">
+        <f t="array" ref="B20">_xll.qlMakeSchedule($B$17,$B$18,"1y",,$B$4,"Following",,"Backward")</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R20C2Schedule,A</v>
+      </c>
+      <c r="L20" s="1"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="4" t="str" cm="1">
+        <f t="array" ref="B21">_xll.qlMakeSchedule($B$17,$B$18,"3m",,$B$4,"Following",,"Backward")</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R21C2Schedule,A</v>
+      </c>
+      <c r="L21" s="1"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L22" s="1"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="2">
+        <v>0.04</v>
+      </c>
+      <c r="L23" s="1"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="L24" s="1"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L25" s="1"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="4" t="str" cm="1">
+        <f t="array" ref="B26">_xll.qlVanillaSwap("Payer",10000,$B$20,$B$23,$B$24,$B$21,$B$11,0,"act/360")</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R26C2VanillaSwap,A</v>
+      </c>
+      <c r="L26" s="1"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L27" s="1"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" s="4" t="str" cm="1">
+        <f t="array" ref="B28">_xll.qlBermudanExercise(Q5:Q9)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R28C2BermudanExercise,A</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>90</v>
+      </c>
+      <c r="B30" s="4" t="str" cm="1">
+        <f t="array" ref="B30">_xll.qlSwaption($B$26,_xll.qlEuropeanExercise(Q5))</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R30C2Swaption,A</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" s="4" t="str" cm="1">
+        <f t="array" ref="B31">_xll.qlSwaption($B$26,_xll.qlEuropeanExercise(Q6))</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R31C2Swaption,A</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>92</v>
+      </c>
+      <c r="B32" s="4" t="str" cm="1">
+        <f t="array" ref="B32">_xll.qlSwaption($B$26,_xll.qlEuropeanExercise(Q7))</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R32C2Swaption,A</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>93</v>
+      </c>
+      <c r="B33" s="4" t="str" cm="1">
+        <f t="array" ref="B33">_xll.qlSwaption($B$26,_xll.qlEuropeanExercise(Q8))</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R33C2Swaption,A</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>94</v>
+      </c>
+      <c r="B34" s="4" t="str" cm="1">
+        <f t="array" ref="B34">_xll.qlSwaption($B$26,_xll.qlEuropeanExercise(Q9))</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R34C2Swaption,A</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>27</v>
+      </c>
+      <c r="B36" s="4" t="str" cm="1">
+        <f t="array" ref="B36">_xll.qlSwaption(B26,B28)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R36C2Swaption,A</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B37" s="4"/>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B38" s="4"/>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>108</v>
+      </c>
+      <c r="B39" s="16">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>96</v>
+      </c>
+      <c r="B40" s="4" t="str" cm="1">
+        <f t="array" ref="B40">_xll.qlGsr(B7,Q5:Q9,U5:U10,V5:V10)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R40C2Gsr,A</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>97</v>
+      </c>
+      <c r="B41" s="4" t="str" cm="1">
+        <f t="array" ref="B41">_xll.qlGaussian1dSwaptionEngine(B40)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R41C2Gaussian1dSwaptionEngine,A</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>99</v>
+      </c>
+      <c r="B43" s="4" t="str" cm="1">
+        <f t="array" ref="B43">_xll.qlLevenbergMarquardt(,,,,T5:T9)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R43C2LevenbergMarquardt,O</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>56</v>
+      </c>
+      <c r="B45">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>57</v>
+      </c>
+      <c r="B46">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>58</v>
+      </c>
+      <c r="B47" s="11">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>59</v>
+      </c>
+      <c r="B48" s="11">
+        <v>1.0000000000000001E-5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>60</v>
+      </c>
+      <c r="B49" s="11">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>100</v>
+      </c>
+      <c r="B50" s="4" t="str" cm="1">
+        <f t="array" ref="B50">_xll.qlEndCriteria(B45,B46,B47,B48,B49,T5:T9)</f>
+        <v>⚡[test_gaussian1dmodel.xlsx]Bermudan Swaption!R50C2EndCriteria,P</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>105</v>
+      </c>
+      <c r="B52" t="b" cm="1">
+        <f t="array" ref="B52">_xll.qlGsrCalibrateVolatilitiesIterative(B40,T5:T9,B43,B50,,,W5:W9)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B54" s="12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>90</v>
+      </c>
+      <c r="B55" s="17" cm="1">
+        <f t="array" ref="B55">_xll.qlInstrumentNPV(B30,_xll.qlInstrumentSetPricingEngine(B30,$B$41,$B$52))</f>
+        <v>21.703395415539141</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>91</v>
+      </c>
+      <c r="B56" s="17" cm="1">
+        <f t="array" ref="B56">_xll.qlInstrumentNPV(B31,_xll.qlInstrumentSetPricingEngine(B31,$B$41,$B$52))</f>
+        <v>96.520281949812968</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>92</v>
+      </c>
+      <c r="B57" s="17" cm="1">
+        <f t="array" ref="B57">_xll.qlInstrumentNPV(B32,_xll.qlInstrumentSetPricingEngine(B32,$B$41,$B$52))</f>
+        <v>123.61092110727894</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>93</v>
+      </c>
+      <c r="B58" s="17" cm="1">
+        <f t="array" ref="B58">_xll.qlInstrumentNPV(B33,_xll.qlInstrumentSetPricingEngine(B33,$B$41,$B$52))</f>
+        <v>110.3399969979758</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>94</v>
+      </c>
+      <c r="B59" s="17" cm="1">
+        <f t="array" ref="B59">_xll.qlInstrumentNPV(B34,_xll.qlInstrumentSetPricingEngine(B34,$B$41,$B$52))</f>
+        <v>67.704758683644968</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>27</v>
+      </c>
+      <c r="B61" s="17" cm="1">
+        <f t="array" ref="B61">_xll.qlInstrumentNPV(B36,_xll.qlInstrumentSetPricingEngine(B36,$B$41,$B$52))</f>
+        <v>177.75574893499586</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>107</v>
+      </c>
+      <c r="B62" s="17">
+        <f>B61-MAX(B55:B59)</f>
+        <v>54.144827827716924</v>
       </c>
     </row>
   </sheetData>

</xml_diff>